<commit_message>
Changing Dataschema in P1 and P2 to ISCED-2011 Standard
</commit_message>
<xml_diff>
--- a/rmonize/data_schema/Dataschema_P1.xlsx
+++ b/rmonize/data_schema/Dataschema_P1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20416"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\use-cases-harmonisation\rmonize\data_schema\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schwarz-f\Desktop\use-cases-harmonisation\rmonize\data_schema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF108BD9-EC6D-4B81-9906-F93C9804C1FC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DBE91B7-173A-4B3C-BD29-E3D3E1F04F4A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="286">
   <si>
     <t>index</t>
   </si>
@@ -763,24 +763,6 @@
     <t>female</t>
   </si>
   <si>
-    <t>none</t>
-  </si>
-  <si>
-    <t>primary school completed</t>
-  </si>
-  <si>
-    <t>technical/professional school completed</t>
-  </si>
-  <si>
-    <t>secondary school</t>
-  </si>
-  <si>
-    <t>longer education (incl. university)</t>
-  </si>
-  <si>
-    <t>not specified</t>
-  </si>
-  <si>
     <t>never</t>
   </si>
   <si>
@@ -875,6 +857,36 @@
   </si>
   <si>
     <t>Body Mass Index at baseline [kg/m²]</t>
+  </si>
+  <si>
+    <t>Early Childhood Education</t>
+  </si>
+  <si>
+    <t>Primary Education</t>
+  </si>
+  <si>
+    <t>Lower Secondary Education</t>
+  </si>
+  <si>
+    <t>Upper Secondary Education</t>
+  </si>
+  <si>
+    <t>Post-secondary non-tertiary education</t>
+  </si>
+  <si>
+    <t>Short-Cycle Tertiary Education</t>
+  </si>
+  <si>
+    <t>Bachelor's or equivalent level</t>
+  </si>
+  <si>
+    <t>Master's or equivalent level</t>
+  </si>
+  <si>
+    <t>Doctoral or equivalent level</t>
+  </si>
+  <si>
+    <t>Other</t>
   </si>
 </sst>
 </file>
@@ -929,9 +941,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Normal 4" xfId="1" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -947,7 +959,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1244,7 +1256,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D129"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625"/>
     <col min="2" max="2" width="34.140625" bestFit="1" customWidth="1"/>
@@ -1271,10 +1283,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="C2" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="D2" t="s">
         <v>4</v>
@@ -1302,7 +1314,7 @@
         <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
@@ -1330,7 +1342,7 @@
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>
@@ -1358,7 +1370,7 @@
         <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
@@ -1736,7 +1748,7 @@
         <v>67</v>
       </c>
       <c r="C35" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="D35" t="s">
         <v>11</v>
@@ -1750,7 +1762,7 @@
         <v>68</v>
       </c>
       <c r="C36" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="D36" t="s">
         <v>11</v>
@@ -1792,7 +1804,7 @@
         <v>73</v>
       </c>
       <c r="C39" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="D39" t="s">
         <v>11</v>
@@ -1820,7 +1832,7 @@
         <v>76</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="D41" t="s">
         <v>11</v>
@@ -1932,7 +1944,7 @@
         <v>91</v>
       </c>
       <c r="C49" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="D49" t="s">
         <v>11</v>
@@ -2072,7 +2084,7 @@
         <v>110</v>
       </c>
       <c r="C59" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="D59" t="s">
         <v>11</v>
@@ -2086,7 +2098,7 @@
         <v>111</v>
       </c>
       <c r="C60" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="D60" t="s">
         <v>11</v>
@@ -2212,7 +2224,7 @@
         <v>128</v>
       </c>
       <c r="C69" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="D69" t="s">
         <v>11</v>
@@ -2240,7 +2252,7 @@
         <v>131</v>
       </c>
       <c r="C71" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="D71" t="s">
         <v>11</v>
@@ -2408,7 +2420,7 @@
         <v>154</v>
       </c>
       <c r="C83" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="D83" t="s">
         <v>11</v>
@@ -2506,7 +2518,7 @@
         <v>167</v>
       </c>
       <c r="C90" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="D90" t="s">
         <v>11</v>
@@ -2898,7 +2910,7 @@
         <v>222</v>
       </c>
       <c r="C118" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="D118" t="s">
         <v>11</v>
@@ -2940,7 +2952,7 @@
         <v>227</v>
       </c>
       <c r="C121" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="D121" t="s">
         <v>11</v>
@@ -3038,7 +3050,7 @@
         <v>240</v>
       </c>
       <c r="C128" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="D128" t="s">
         <v>11</v>
@@ -3049,10 +3061,10 @@
         <v>128</v>
       </c>
       <c r="B129" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="C129" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="D129" t="s">
         <v>4</v>
@@ -3073,8 +3085,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C64"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C68"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="51.28515625" bestFit="1" customWidth="1"/>
@@ -3119,7 +3131,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>244</v>
+        <v>276</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -3130,7 +3142,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>245</v>
+        <v>277</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -3141,7 +3153,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>246</v>
+        <v>278</v>
       </c>
       <c r="C6">
         <v>2</v>
@@ -3152,7 +3164,7 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>247</v>
+        <v>279</v>
       </c>
       <c r="C7">
         <v>3</v>
@@ -3163,7 +3175,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>248</v>
+        <v>280</v>
       </c>
       <c r="C8">
         <v>4</v>
@@ -3174,7 +3186,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>249</v>
+        <v>281</v>
       </c>
       <c r="C9">
         <v>5</v>
@@ -3182,126 +3194,170 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>250</v>
+        <v>282</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>251</v>
+        <v>283</v>
       </c>
       <c r="C11">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>252</v>
+        <v>284</v>
       </c>
       <c r="C12">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>253</v>
+        <v>285</v>
       </c>
       <c r="C13">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>256</v>
+        <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>258</v>
+        <v>244</v>
       </c>
       <c r="C14">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>256</v>
+        <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>278</v>
+        <v>245</v>
       </c>
       <c r="C15">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>256</v>
+        <v>12</v>
       </c>
       <c r="B16" t="s">
-        <v>275</v>
+        <v>246</v>
       </c>
       <c r="C16">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>256</v>
+        <v>12</v>
       </c>
       <c r="B17" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
       <c r="C17">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="B18" t="s">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="C18">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="B19" t="s">
-        <v>260</v>
+        <v>272</v>
       </c>
       <c r="C19">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="B20" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="C20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>250</v>
+      </c>
+      <c r="B21" t="s">
+        <v>253</v>
+      </c>
+      <c r="C21">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>250</v>
+      </c>
+      <c r="B22" t="s">
+        <v>255</v>
+      </c>
+      <c r="C22">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>250</v>
+      </c>
+      <c r="B23" t="s">
+        <v>254</v>
+      </c>
+      <c r="C23">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>250</v>
+      </c>
+      <c r="B24" t="s">
+        <v>270</v>
+      </c>
+      <c r="C24">
         <v>6</v>
       </c>
     </row>
-    <row r="64" ht="14.1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="68" ht="14.1" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <customSheetViews>
     <customSheetView guid="{85760D7C-312A-4647-B300-A227B229A527}">
@@ -3316,15 +3372,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Zeit xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413" xsi:nil="true"/>
@@ -3334,6 +3381,15 @@
     <TaxCatchAll xmlns="12535b08-222e-45d2-b6db-15019f1afee6" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3578,14 +3634,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EBBE8B2F-371B-4499-AB2D-BE5C88E1FE7D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0EB6D834-F5F1-4875-9BFF-E74D4F6F598A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
@@ -3598,6 +3646,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="12535b08-222e-45d2-b6db-15019f1afee6"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EBBE8B2F-371B-4499-AB2D-BE5C88E1FE7D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
added reference to ISCED 2011 in the variables description of the Dataschema
</commit_message>
<xml_diff>
--- a/rmonize/data_schema/Dataschema_P1.xlsx
+++ b/rmonize/data_schema/Dataschema_P1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schwarz-f\Desktop\use-cases-harmonisation\rmonize\data_schema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DBE91B7-173A-4B3C-BD29-E3D3E1F04F4A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C5138F8-0C10-4C96-A966-A88556A7E43C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
@@ -58,9 +58,6 @@
     <t>EDU_LEVEL</t>
   </si>
   <si>
-    <t>Education</t>
-  </si>
-  <si>
     <t>TOT_PA_QX</t>
   </si>
   <si>
@@ -887,6 +884,9 @@
   </si>
   <si>
     <t>Other</t>
+  </si>
+  <si>
+    <t>Highest level of education [ISCED 2011]</t>
   </si>
 </sst>
 </file>
@@ -1283,10 +1283,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>247</v>
+      </c>
+      <c r="C2" t="s">
         <v>248</v>
-      </c>
-      <c r="C2" t="s">
-        <v>249</v>
       </c>
       <c r="D2" t="s">
         <v>4</v>
@@ -1314,10 +1314,10 @@
         <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1328,7 +1328,7 @@
         <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>285</v>
       </c>
       <c r="D5" t="s">
         <v>4</v>
@@ -1339,13 +1339,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1353,10 +1353,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s">
         <v>12</v>
-      </c>
-      <c r="C7" t="s">
-        <v>13</v>
       </c>
       <c r="D7" t="s">
         <v>4</v>
@@ -1367,13 +1367,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1381,13 +1381,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
         <v>15</v>
       </c>
-      <c r="C9" t="s">
-        <v>16</v>
-      </c>
       <c r="D9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1395,13 +1395,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" t="s">
         <v>17</v>
       </c>
-      <c r="C10" t="s">
-        <v>18</v>
-      </c>
       <c r="D10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1409,13 +1409,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" t="s">
         <v>19</v>
       </c>
-      <c r="C11" t="s">
-        <v>20</v>
-      </c>
       <c r="D11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -1423,13 +1423,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" t="s">
         <v>21</v>
       </c>
-      <c r="C12" t="s">
-        <v>22</v>
-      </c>
       <c r="D12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -1437,13 +1437,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" t="s">
         <v>23</v>
       </c>
-      <c r="C13" t="s">
-        <v>24</v>
-      </c>
       <c r="D13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -1451,13 +1451,13 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" t="s">
         <v>25</v>
       </c>
-      <c r="C14" t="s">
-        <v>26</v>
-      </c>
       <c r="D14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -1465,13 +1465,13 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" t="s">
         <v>27</v>
       </c>
-      <c r="C15" t="s">
-        <v>28</v>
-      </c>
       <c r="D15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -1479,13 +1479,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" t="s">
         <v>29</v>
       </c>
-      <c r="C16" t="s">
-        <v>30</v>
-      </c>
       <c r="D16" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -1493,13 +1493,13 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" t="s">
         <v>31</v>
       </c>
-      <c r="C17" t="s">
-        <v>32</v>
-      </c>
       <c r="D17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -1507,13 +1507,13 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" t="s">
         <v>33</v>
       </c>
-      <c r="C18" t="s">
-        <v>34</v>
-      </c>
       <c r="D18" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -1521,13 +1521,13 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
+        <v>34</v>
+      </c>
+      <c r="C19" t="s">
         <v>35</v>
       </c>
-      <c r="C19" t="s">
-        <v>36</v>
-      </c>
       <c r="D19" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -1535,13 +1535,13 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
+        <v>36</v>
+      </c>
+      <c r="C20" t="s">
         <v>37</v>
       </c>
-      <c r="C20" t="s">
-        <v>38</v>
-      </c>
       <c r="D20" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -1549,13 +1549,13 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" t="s">
         <v>39</v>
       </c>
-      <c r="C21" t="s">
-        <v>40</v>
-      </c>
       <c r="D21" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -1563,13 +1563,13 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
+        <v>40</v>
+      </c>
+      <c r="C22" t="s">
         <v>41</v>
       </c>
-      <c r="C22" t="s">
-        <v>42</v>
-      </c>
       <c r="D22" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -1577,13 +1577,13 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
+        <v>42</v>
+      </c>
+      <c r="C23" t="s">
         <v>43</v>
       </c>
-      <c r="C23" t="s">
-        <v>44</v>
-      </c>
       <c r="D23" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -1591,13 +1591,13 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
+        <v>44</v>
+      </c>
+      <c r="C24" t="s">
         <v>45</v>
       </c>
-      <c r="C24" t="s">
-        <v>46</v>
-      </c>
       <c r="D24" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -1605,13 +1605,13 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
+        <v>46</v>
+      </c>
+      <c r="C25" t="s">
         <v>47</v>
       </c>
-      <c r="C25" t="s">
-        <v>48</v>
-      </c>
       <c r="D25" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -1619,13 +1619,13 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
+        <v>48</v>
+      </c>
+      <c r="C26" t="s">
         <v>49</v>
       </c>
-      <c r="C26" t="s">
-        <v>50</v>
-      </c>
       <c r="D26" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -1633,13 +1633,13 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
+        <v>50</v>
+      </c>
+      <c r="C27" t="s">
         <v>51</v>
       </c>
-      <c r="C27" t="s">
-        <v>52</v>
-      </c>
       <c r="D27" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -1647,13 +1647,13 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
+        <v>52</v>
+      </c>
+      <c r="C28" t="s">
         <v>53</v>
       </c>
-      <c r="C28" t="s">
-        <v>54</v>
-      </c>
       <c r="D28" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -1661,13 +1661,13 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
+        <v>54</v>
+      </c>
+      <c r="C29" t="s">
         <v>55</v>
       </c>
-      <c r="C29" t="s">
-        <v>56</v>
-      </c>
       <c r="D29" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -1675,13 +1675,13 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
+        <v>56</v>
+      </c>
+      <c r="C30" t="s">
         <v>57</v>
       </c>
-      <c r="C30" t="s">
-        <v>58</v>
-      </c>
       <c r="D30" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -1689,13 +1689,13 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
+        <v>58</v>
+      </c>
+      <c r="C31" t="s">
         <v>59</v>
       </c>
-      <c r="C31" t="s">
-        <v>60</v>
-      </c>
       <c r="D31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -1703,13 +1703,13 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
+        <v>60</v>
+      </c>
+      <c r="C32" t="s">
         <v>61</v>
       </c>
-      <c r="C32" t="s">
-        <v>62</v>
-      </c>
       <c r="D32" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -1717,13 +1717,13 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
+        <v>62</v>
+      </c>
+      <c r="C33" t="s">
         <v>63</v>
       </c>
-      <c r="C33" t="s">
-        <v>64</v>
-      </c>
       <c r="D33" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -1731,13 +1731,13 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
+        <v>64</v>
+      </c>
+      <c r="C34" t="s">
         <v>65</v>
       </c>
-      <c r="C34" t="s">
-        <v>66</v>
-      </c>
       <c r="D34" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -1745,13 +1745,13 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C35" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D35" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -1759,13 +1759,13 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C36" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D36" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -1773,13 +1773,13 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
+        <v>68</v>
+      </c>
+      <c r="C37" t="s">
         <v>69</v>
       </c>
-      <c r="C37" t="s">
-        <v>70</v>
-      </c>
       <c r="D37" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -1787,13 +1787,13 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
+        <v>70</v>
+      </c>
+      <c r="C38" t="s">
         <v>71</v>
       </c>
-      <c r="C38" t="s">
-        <v>72</v>
-      </c>
       <c r="D38" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -1801,13 +1801,13 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C39" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D39" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -1815,13 +1815,13 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
+        <v>73</v>
+      </c>
+      <c r="C40" t="s">
         <v>74</v>
       </c>
-      <c r="C40" t="s">
-        <v>75</v>
-      </c>
       <c r="D40" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -1829,13 +1829,13 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D41" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -1843,13 +1843,13 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
+        <v>76</v>
+      </c>
+      <c r="C42" t="s">
         <v>77</v>
       </c>
-      <c r="C42" t="s">
-        <v>78</v>
-      </c>
       <c r="D42" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -1857,13 +1857,13 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
+        <v>78</v>
+      </c>
+      <c r="C43" t="s">
         <v>79</v>
       </c>
-      <c r="C43" t="s">
-        <v>80</v>
-      </c>
       <c r="D43" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -1871,13 +1871,13 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
+        <v>80</v>
+      </c>
+      <c r="C44" t="s">
         <v>81</v>
       </c>
-      <c r="C44" t="s">
-        <v>82</v>
-      </c>
       <c r="D44" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -1885,13 +1885,13 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
+        <v>82</v>
+      </c>
+      <c r="C45" t="s">
         <v>83</v>
       </c>
-      <c r="C45" t="s">
-        <v>84</v>
-      </c>
       <c r="D45" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
@@ -1899,13 +1899,13 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
+        <v>84</v>
+      </c>
+      <c r="C46" t="s">
         <v>85</v>
       </c>
-      <c r="C46" t="s">
-        <v>86</v>
-      </c>
       <c r="D46" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -1913,13 +1913,13 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
+        <v>86</v>
+      </c>
+      <c r="C47" t="s">
         <v>87</v>
       </c>
-      <c r="C47" t="s">
-        <v>88</v>
-      </c>
       <c r="D47" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -1927,13 +1927,13 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
+        <v>88</v>
+      </c>
+      <c r="C48" t="s">
         <v>89</v>
       </c>
-      <c r="C48" t="s">
-        <v>90</v>
-      </c>
       <c r="D48" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -1941,13 +1941,13 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C49" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D49" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -1955,13 +1955,13 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
+        <v>91</v>
+      </c>
+      <c r="C50" t="s">
         <v>92</v>
       </c>
-      <c r="C50" t="s">
-        <v>93</v>
-      </c>
       <c r="D50" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -1969,13 +1969,13 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
+        <v>93</v>
+      </c>
+      <c r="C51" t="s">
         <v>94</v>
       </c>
-      <c r="C51" t="s">
-        <v>95</v>
-      </c>
       <c r="D51" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -1983,13 +1983,13 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
+        <v>95</v>
+      </c>
+      <c r="C52" t="s">
         <v>96</v>
       </c>
-      <c r="C52" t="s">
-        <v>97</v>
-      </c>
       <c r="D52" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -1997,13 +1997,13 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
+        <v>97</v>
+      </c>
+      <c r="C53" t="s">
         <v>98</v>
       </c>
-      <c r="C53" t="s">
-        <v>99</v>
-      </c>
       <c r="D53" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
@@ -2011,13 +2011,13 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
+        <v>99</v>
+      </c>
+      <c r="C54" t="s">
         <v>100</v>
       </c>
-      <c r="C54" t="s">
-        <v>101</v>
-      </c>
       <c r="D54" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -2025,13 +2025,13 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
+        <v>101</v>
+      </c>
+      <c r="C55" t="s">
         <v>102</v>
       </c>
-      <c r="C55" t="s">
-        <v>103</v>
-      </c>
       <c r="D55" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -2039,13 +2039,13 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
+        <v>103</v>
+      </c>
+      <c r="C56" t="s">
         <v>104</v>
       </c>
-      <c r="C56" t="s">
-        <v>105</v>
-      </c>
       <c r="D56" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -2053,13 +2053,13 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
+        <v>105</v>
+      </c>
+      <c r="C57" t="s">
         <v>106</v>
       </c>
-      <c r="C57" t="s">
-        <v>107</v>
-      </c>
       <c r="D57" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -2067,13 +2067,13 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
+        <v>107</v>
+      </c>
+      <c r="C58" t="s">
         <v>108</v>
       </c>
-      <c r="C58" t="s">
-        <v>109</v>
-      </c>
       <c r="D58" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -2081,13 +2081,13 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C59" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D59" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -2095,13 +2095,13 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C60" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D60" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -2109,13 +2109,13 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
+        <v>111</v>
+      </c>
+      <c r="C61" t="s">
         <v>112</v>
       </c>
-      <c r="C61" t="s">
-        <v>113</v>
-      </c>
       <c r="D61" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -2123,13 +2123,13 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
+        <v>113</v>
+      </c>
+      <c r="C62" t="s">
         <v>114</v>
       </c>
-      <c r="C62" t="s">
-        <v>115</v>
-      </c>
       <c r="D62" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -2137,13 +2137,13 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
+        <v>115</v>
+      </c>
+      <c r="C63" t="s">
         <v>116</v>
       </c>
-      <c r="C63" t="s">
-        <v>117</v>
-      </c>
       <c r="D63" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
@@ -2151,13 +2151,13 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
+        <v>117</v>
+      </c>
+      <c r="C64" t="s">
         <v>118</v>
       </c>
-      <c r="C64" t="s">
-        <v>119</v>
-      </c>
       <c r="D64" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
@@ -2165,13 +2165,13 @@
         <v>64</v>
       </c>
       <c r="B65" t="s">
+        <v>119</v>
+      </c>
+      <c r="C65" t="s">
         <v>120</v>
       </c>
-      <c r="C65" t="s">
-        <v>121</v>
-      </c>
       <c r="D65" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
@@ -2179,13 +2179,13 @@
         <v>65</v>
       </c>
       <c r="B66" t="s">
+        <v>121</v>
+      </c>
+      <c r="C66" t="s">
         <v>122</v>
       </c>
-      <c r="C66" t="s">
-        <v>123</v>
-      </c>
       <c r="D66" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -2193,13 +2193,13 @@
         <v>66</v>
       </c>
       <c r="B67" t="s">
+        <v>123</v>
+      </c>
+      <c r="C67" t="s">
         <v>124</v>
       </c>
-      <c r="C67" t="s">
-        <v>125</v>
-      </c>
       <c r="D67" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -2207,13 +2207,13 @@
         <v>67</v>
       </c>
       <c r="B68" t="s">
+        <v>125</v>
+      </c>
+      <c r="C68" t="s">
         <v>126</v>
       </c>
-      <c r="C68" t="s">
-        <v>127</v>
-      </c>
       <c r="D68" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -2221,13 +2221,13 @@
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C69" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D69" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
@@ -2235,13 +2235,13 @@
         <v>69</v>
       </c>
       <c r="B70" t="s">
+        <v>128</v>
+      </c>
+      <c r="C70" t="s">
         <v>129</v>
       </c>
-      <c r="C70" t="s">
-        <v>130</v>
-      </c>
       <c r="D70" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
@@ -2249,13 +2249,13 @@
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C71" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D71" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
@@ -2263,13 +2263,13 @@
         <v>71</v>
       </c>
       <c r="B72" t="s">
+        <v>131</v>
+      </c>
+      <c r="C72" t="s">
         <v>132</v>
       </c>
-      <c r="C72" t="s">
-        <v>133</v>
-      </c>
       <c r="D72" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -2277,13 +2277,13 @@
         <v>72</v>
       </c>
       <c r="B73" t="s">
+        <v>133</v>
+      </c>
+      <c r="C73" t="s">
         <v>134</v>
       </c>
-      <c r="C73" t="s">
-        <v>135</v>
-      </c>
       <c r="D73" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
@@ -2291,13 +2291,13 @@
         <v>73</v>
       </c>
       <c r="B74" t="s">
+        <v>135</v>
+      </c>
+      <c r="C74" t="s">
         <v>136</v>
       </c>
-      <c r="C74" t="s">
-        <v>137</v>
-      </c>
       <c r="D74" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
@@ -2305,13 +2305,13 @@
         <v>74</v>
       </c>
       <c r="B75" t="s">
+        <v>137</v>
+      </c>
+      <c r="C75" t="s">
         <v>138</v>
       </c>
-      <c r="C75" t="s">
-        <v>139</v>
-      </c>
       <c r="D75" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -2319,13 +2319,13 @@
         <v>75</v>
       </c>
       <c r="B76" t="s">
+        <v>139</v>
+      </c>
+      <c r="C76" t="s">
         <v>140</v>
       </c>
-      <c r="C76" t="s">
-        <v>141</v>
-      </c>
       <c r="D76" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -2333,13 +2333,13 @@
         <v>76</v>
       </c>
       <c r="B77" t="s">
+        <v>141</v>
+      </c>
+      <c r="C77" t="s">
         <v>142</v>
       </c>
-      <c r="C77" t="s">
-        <v>143</v>
-      </c>
       <c r="D77" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
@@ -2347,13 +2347,13 @@
         <v>77</v>
       </c>
       <c r="B78" t="s">
+        <v>143</v>
+      </c>
+      <c r="C78" t="s">
         <v>144</v>
       </c>
-      <c r="C78" t="s">
-        <v>145</v>
-      </c>
       <c r="D78" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
@@ -2361,13 +2361,13 @@
         <v>78</v>
       </c>
       <c r="B79" t="s">
+        <v>145</v>
+      </c>
+      <c r="C79" t="s">
         <v>146</v>
       </c>
-      <c r="C79" t="s">
-        <v>147</v>
-      </c>
       <c r="D79" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
@@ -2375,13 +2375,13 @@
         <v>79</v>
       </c>
       <c r="B80" t="s">
+        <v>147</v>
+      </c>
+      <c r="C80" t="s">
         <v>148</v>
       </c>
-      <c r="C80" t="s">
-        <v>149</v>
-      </c>
       <c r="D80" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
@@ -2389,13 +2389,13 @@
         <v>80</v>
       </c>
       <c r="B81" t="s">
+        <v>149</v>
+      </c>
+      <c r="C81" t="s">
         <v>150</v>
       </c>
-      <c r="C81" t="s">
-        <v>151</v>
-      </c>
       <c r="D81" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
@@ -2403,13 +2403,13 @@
         <v>81</v>
       </c>
       <c r="B82" t="s">
+        <v>151</v>
+      </c>
+      <c r="C82" t="s">
         <v>152</v>
       </c>
-      <c r="C82" t="s">
-        <v>153</v>
-      </c>
       <c r="D82" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
@@ -2417,13 +2417,13 @@
         <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C83" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D83" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
@@ -2431,13 +2431,13 @@
         <v>83</v>
       </c>
       <c r="B84" t="s">
+        <v>154</v>
+      </c>
+      <c r="C84" t="s">
         <v>155</v>
       </c>
-      <c r="C84" t="s">
-        <v>156</v>
-      </c>
       <c r="D84" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
@@ -2445,13 +2445,13 @@
         <v>84</v>
       </c>
       <c r="B85" t="s">
+        <v>156</v>
+      </c>
+      <c r="C85" t="s">
         <v>157</v>
       </c>
-      <c r="C85" t="s">
-        <v>158</v>
-      </c>
       <c r="D85" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
@@ -2459,13 +2459,13 @@
         <v>85</v>
       </c>
       <c r="B86" t="s">
+        <v>158</v>
+      </c>
+      <c r="C86" t="s">
         <v>159</v>
       </c>
-      <c r="C86" t="s">
-        <v>160</v>
-      </c>
       <c r="D86" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
@@ -2473,13 +2473,13 @@
         <v>86</v>
       </c>
       <c r="B87" t="s">
+        <v>160</v>
+      </c>
+      <c r="C87" t="s">
         <v>161</v>
       </c>
-      <c r="C87" t="s">
-        <v>162</v>
-      </c>
       <c r="D87" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
@@ -2487,13 +2487,13 @@
         <v>87</v>
       </c>
       <c r="B88" t="s">
+        <v>162</v>
+      </c>
+      <c r="C88" t="s">
         <v>163</v>
       </c>
-      <c r="C88" t="s">
-        <v>164</v>
-      </c>
       <c r="D88" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
@@ -2501,13 +2501,13 @@
         <v>88</v>
       </c>
       <c r="B89" t="s">
+        <v>164</v>
+      </c>
+      <c r="C89" t="s">
         <v>165</v>
       </c>
-      <c r="C89" t="s">
-        <v>166</v>
-      </c>
       <c r="D89" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
@@ -2515,13 +2515,13 @@
         <v>89</v>
       </c>
       <c r="B90" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C90" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D90" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
@@ -2529,13 +2529,13 @@
         <v>90</v>
       </c>
       <c r="B91" t="s">
+        <v>167</v>
+      </c>
+      <c r="C91" t="s">
         <v>168</v>
       </c>
-      <c r="C91" t="s">
-        <v>169</v>
-      </c>
       <c r="D91" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
@@ -2543,13 +2543,13 @@
         <v>91</v>
       </c>
       <c r="B92" t="s">
+        <v>169</v>
+      </c>
+      <c r="C92" t="s">
         <v>170</v>
       </c>
-      <c r="C92" t="s">
-        <v>171</v>
-      </c>
       <c r="D92" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
@@ -2557,13 +2557,13 @@
         <v>92</v>
       </c>
       <c r="B93" t="s">
+        <v>171</v>
+      </c>
+      <c r="C93" t="s">
         <v>172</v>
       </c>
-      <c r="C93" t="s">
-        <v>173</v>
-      </c>
       <c r="D93" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
@@ -2571,13 +2571,13 @@
         <v>93</v>
       </c>
       <c r="B94" t="s">
+        <v>173</v>
+      </c>
+      <c r="C94" t="s">
         <v>174</v>
       </c>
-      <c r="C94" t="s">
-        <v>175</v>
-      </c>
       <c r="D94" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
@@ -2585,13 +2585,13 @@
         <v>94</v>
       </c>
       <c r="B95" t="s">
+        <v>175</v>
+      </c>
+      <c r="C95" t="s">
         <v>176</v>
       </c>
-      <c r="C95" t="s">
-        <v>177</v>
-      </c>
       <c r="D95" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
@@ -2599,13 +2599,13 @@
         <v>95</v>
       </c>
       <c r="B96" t="s">
+        <v>177</v>
+      </c>
+      <c r="C96" t="s">
         <v>178</v>
       </c>
-      <c r="C96" t="s">
-        <v>179</v>
-      </c>
       <c r="D96" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
@@ -2613,13 +2613,13 @@
         <v>96</v>
       </c>
       <c r="B97" t="s">
+        <v>179</v>
+      </c>
+      <c r="C97" t="s">
         <v>180</v>
       </c>
-      <c r="C97" t="s">
-        <v>181</v>
-      </c>
       <c r="D97" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
@@ -2627,13 +2627,13 @@
         <v>97</v>
       </c>
       <c r="B98" t="s">
+        <v>181</v>
+      </c>
+      <c r="C98" t="s">
         <v>182</v>
       </c>
-      <c r="C98" t="s">
-        <v>183</v>
-      </c>
       <c r="D98" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
@@ -2641,13 +2641,13 @@
         <v>98</v>
       </c>
       <c r="B99" t="s">
+        <v>183</v>
+      </c>
+      <c r="C99" t="s">
         <v>184</v>
       </c>
-      <c r="C99" t="s">
-        <v>185</v>
-      </c>
       <c r="D99" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
@@ -2655,13 +2655,13 @@
         <v>99</v>
       </c>
       <c r="B100" t="s">
+        <v>185</v>
+      </c>
+      <c r="C100" t="s">
         <v>186</v>
       </c>
-      <c r="C100" t="s">
-        <v>187</v>
-      </c>
       <c r="D100" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
@@ -2669,13 +2669,13 @@
         <v>100</v>
       </c>
       <c r="B101" t="s">
+        <v>187</v>
+      </c>
+      <c r="C101" t="s">
         <v>188</v>
       </c>
-      <c r="C101" t="s">
-        <v>189</v>
-      </c>
       <c r="D101" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
@@ -2683,13 +2683,13 @@
         <v>101</v>
       </c>
       <c r="B102" t="s">
+        <v>189</v>
+      </c>
+      <c r="C102" t="s">
         <v>190</v>
       </c>
-      <c r="C102" t="s">
-        <v>191</v>
-      </c>
       <c r="D102" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
@@ -2697,13 +2697,13 @@
         <v>102</v>
       </c>
       <c r="B103" t="s">
+        <v>191</v>
+      </c>
+      <c r="C103" t="s">
         <v>192</v>
       </c>
-      <c r="C103" t="s">
-        <v>193</v>
-      </c>
       <c r="D103" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
@@ -2711,13 +2711,13 @@
         <v>103</v>
       </c>
       <c r="B104" t="s">
+        <v>193</v>
+      </c>
+      <c r="C104" t="s">
         <v>194</v>
       </c>
-      <c r="C104" t="s">
-        <v>195</v>
-      </c>
       <c r="D104" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
@@ -2725,13 +2725,13 @@
         <v>104</v>
       </c>
       <c r="B105" t="s">
+        <v>195</v>
+      </c>
+      <c r="C105" t="s">
         <v>196</v>
       </c>
-      <c r="C105" t="s">
-        <v>197</v>
-      </c>
       <c r="D105" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
@@ -2739,13 +2739,13 @@
         <v>105</v>
       </c>
       <c r="B106" t="s">
+        <v>197</v>
+      </c>
+      <c r="C106" t="s">
         <v>198</v>
       </c>
-      <c r="C106" t="s">
-        <v>199</v>
-      </c>
       <c r="D106" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
@@ -2753,13 +2753,13 @@
         <v>106</v>
       </c>
       <c r="B107" t="s">
+        <v>199</v>
+      </c>
+      <c r="C107" t="s">
         <v>200</v>
       </c>
-      <c r="C107" t="s">
-        <v>201</v>
-      </c>
       <c r="D107" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
@@ -2767,13 +2767,13 @@
         <v>107</v>
       </c>
       <c r="B108" t="s">
+        <v>201</v>
+      </c>
+      <c r="C108" t="s">
         <v>202</v>
       </c>
-      <c r="C108" t="s">
-        <v>203</v>
-      </c>
       <c r="D108" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
@@ -2781,13 +2781,13 @@
         <v>108</v>
       </c>
       <c r="B109" t="s">
+        <v>203</v>
+      </c>
+      <c r="C109" t="s">
         <v>204</v>
       </c>
-      <c r="C109" t="s">
-        <v>205</v>
-      </c>
       <c r="D109" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
@@ -2795,13 +2795,13 @@
         <v>109</v>
       </c>
       <c r="B110" t="s">
+        <v>205</v>
+      </c>
+      <c r="C110" t="s">
         <v>206</v>
       </c>
-      <c r="C110" t="s">
-        <v>207</v>
-      </c>
       <c r="D110" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
@@ -2809,13 +2809,13 @@
         <v>110</v>
       </c>
       <c r="B111" t="s">
+        <v>207</v>
+      </c>
+      <c r="C111" t="s">
         <v>208</v>
       </c>
-      <c r="C111" t="s">
-        <v>209</v>
-      </c>
       <c r="D111" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
@@ -2823,13 +2823,13 @@
         <v>111</v>
       </c>
       <c r="B112" t="s">
+        <v>209</v>
+      </c>
+      <c r="C112" t="s">
         <v>210</v>
       </c>
-      <c r="C112" t="s">
-        <v>211</v>
-      </c>
       <c r="D112" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
@@ -2837,13 +2837,13 @@
         <v>112</v>
       </c>
       <c r="B113" t="s">
+        <v>211</v>
+      </c>
+      <c r="C113" t="s">
         <v>212</v>
       </c>
-      <c r="C113" t="s">
-        <v>213</v>
-      </c>
       <c r="D113" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
@@ -2851,13 +2851,13 @@
         <v>113</v>
       </c>
       <c r="B114" t="s">
+        <v>213</v>
+      </c>
+      <c r="C114" t="s">
         <v>214</v>
       </c>
-      <c r="C114" t="s">
-        <v>215</v>
-      </c>
       <c r="D114" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
@@ -2865,13 +2865,13 @@
         <v>114</v>
       </c>
       <c r="B115" t="s">
+        <v>215</v>
+      </c>
+      <c r="C115" t="s">
         <v>216</v>
       </c>
-      <c r="C115" t="s">
-        <v>217</v>
-      </c>
       <c r="D115" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
@@ -2879,13 +2879,13 @@
         <v>115</v>
       </c>
       <c r="B116" t="s">
+        <v>217</v>
+      </c>
+      <c r="C116" t="s">
         <v>218</v>
       </c>
-      <c r="C116" t="s">
-        <v>219</v>
-      </c>
       <c r="D116" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
@@ -2893,13 +2893,13 @@
         <v>116</v>
       </c>
       <c r="B117" t="s">
+        <v>219</v>
+      </c>
+      <c r="C117" t="s">
         <v>220</v>
       </c>
-      <c r="C117" t="s">
-        <v>221</v>
-      </c>
       <c r="D117" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
@@ -2907,13 +2907,13 @@
         <v>117</v>
       </c>
       <c r="B118" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C118" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D118" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
@@ -2921,13 +2921,13 @@
         <v>118</v>
       </c>
       <c r="B119" t="s">
+        <v>222</v>
+      </c>
+      <c r="C119" t="s">
         <v>223</v>
       </c>
-      <c r="C119" t="s">
-        <v>224</v>
-      </c>
       <c r="D119" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
@@ -2935,13 +2935,13 @@
         <v>119</v>
       </c>
       <c r="B120" t="s">
+        <v>224</v>
+      </c>
+      <c r="C120" t="s">
         <v>225</v>
       </c>
-      <c r="C120" t="s">
-        <v>226</v>
-      </c>
       <c r="D120" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
@@ -2949,13 +2949,13 @@
         <v>120</v>
       </c>
       <c r="B121" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C121" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D121" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
@@ -2963,13 +2963,13 @@
         <v>121</v>
       </c>
       <c r="B122" t="s">
+        <v>227</v>
+      </c>
+      <c r="C122" t="s">
         <v>228</v>
       </c>
-      <c r="C122" t="s">
-        <v>229</v>
-      </c>
       <c r="D122" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
@@ -2977,13 +2977,13 @@
         <v>122</v>
       </c>
       <c r="B123" t="s">
+        <v>229</v>
+      </c>
+      <c r="C123" t="s">
         <v>230</v>
       </c>
-      <c r="C123" t="s">
-        <v>231</v>
-      </c>
       <c r="D123" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
@@ -2991,13 +2991,13 @@
         <v>123</v>
       </c>
       <c r="B124" t="s">
+        <v>231</v>
+      </c>
+      <c r="C124" t="s">
         <v>232</v>
       </c>
-      <c r="C124" t="s">
-        <v>233</v>
-      </c>
       <c r="D124" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
@@ -3005,13 +3005,13 @@
         <v>124</v>
       </c>
       <c r="B125" t="s">
+        <v>233</v>
+      </c>
+      <c r="C125" t="s">
         <v>234</v>
       </c>
-      <c r="C125" t="s">
-        <v>235</v>
-      </c>
       <c r="D125" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
@@ -3019,13 +3019,13 @@
         <v>125</v>
       </c>
       <c r="B126" t="s">
+        <v>235</v>
+      </c>
+      <c r="C126" t="s">
         <v>236</v>
       </c>
-      <c r="C126" t="s">
-        <v>237</v>
-      </c>
       <c r="D126" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
@@ -3033,13 +3033,13 @@
         <v>126</v>
       </c>
       <c r="B127" t="s">
+        <v>237</v>
+      </c>
+      <c r="C127" t="s">
         <v>238</v>
       </c>
-      <c r="C127" t="s">
-        <v>239</v>
-      </c>
       <c r="D127" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
@@ -3047,13 +3047,13 @@
         <v>127</v>
       </c>
       <c r="B128" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C128" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D128" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
@@ -3061,10 +3061,10 @@
         <v>128</v>
       </c>
       <c r="B129" t="s">
+        <v>249</v>
+      </c>
+      <c r="C129" t="s">
         <v>250</v>
-      </c>
-      <c r="C129" t="s">
-        <v>251</v>
       </c>
       <c r="D129" t="s">
         <v>4</v>
@@ -3095,7 +3095,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B1" t="s">
         <v>2</v>
@@ -3109,7 +3109,7 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -3120,7 +3120,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C3">
         <v>2</v>
@@ -3131,7 +3131,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -3142,7 +3142,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -3153,7 +3153,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C6">
         <v>2</v>
@@ -3164,7 +3164,7 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C7">
         <v>3</v>
@@ -3175,7 +3175,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C8">
         <v>4</v>
@@ -3186,7 +3186,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C9">
         <v>5</v>
@@ -3197,7 +3197,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C10">
         <v>6</v>
@@ -3208,7 +3208,7 @@
         <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C11">
         <v>7</v>
@@ -3219,7 +3219,7 @@
         <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C12">
         <v>8</v>
@@ -3230,7 +3230,7 @@
         <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C13">
         <v>9</v>
@@ -3238,10 +3238,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -3249,10 +3249,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B15" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C15">
         <v>2</v>
@@ -3260,10 +3260,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C16">
         <v>3</v>
@@ -3271,10 +3271,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B17" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C17">
         <v>4</v>
@@ -3282,10 +3282,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B18" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -3293,10 +3293,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B19" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -3304,10 +3304,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B20" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C20">
         <v>2</v>
@@ -3315,10 +3315,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B21" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C21">
         <v>3</v>
@@ -3326,10 +3326,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B22" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C22">
         <v>4</v>
@@ -3337,10 +3337,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B23" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C23">
         <v>5</v>
@@ -3348,10 +3348,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B24" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C24">
         <v>6</v>
@@ -3372,6 +3372,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Zeit xmlns="b63cdcf7-47fa-43f6-87e5-23b415b5c413" xsi:nil="true"/>
@@ -3381,15 +3390,6 @@
     <TaxCatchAll xmlns="12535b08-222e-45d2-b6db-15019f1afee6" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3634,6 +3634,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EBBE8B2F-371B-4499-AB2D-BE5C88E1FE7D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0EB6D834-F5F1-4875-9BFF-E74D4F6F598A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
@@ -3646,14 +3654,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="12535b08-222e-45d2-b6db-15019f1afee6"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EBBE8B2F-371B-4499-AB2D-BE5C88E1FE7D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>